<commit_message>
Switch to horizontal pin headers
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="125">
   <si>
     <t xml:space="preserve">ESP32S3Board PCS BOM</t>
   </si>
@@ -251,7 +251,10 @@
     <t xml:space="preserve">LED BLUE CLEAR 0402 SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">J1, J3, J4, J5, J6, J7</t>
+    <t xml:space="preserve">J1, J3, J4, J5, J6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THT</t>
   </si>
   <si>
     <t xml:space="preserve">not fitted</t>
@@ -272,7 +275,7 @@
     <t xml:space="preserve">SMD/THT</t>
   </si>
   <si>
-    <t xml:space="preserve">J8</t>
+    <t xml:space="preserve">J7</t>
   </si>
   <si>
     <t xml:space="preserve">JST Sales America Inc.</t>
@@ -285,6 +288,9 @@
   </si>
   <si>
     <t xml:space="preserve">4-SMD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP1</t>
   </si>
   <si>
     <t xml:space="preserve">L1</t>
@@ -481,7 +487,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -536,28 +542,15 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -622,7 +615,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -647,40 +640,28 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -766,9 +747,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>655560</xdr:colOff>
+      <xdr:colOff>654840</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>147960</xdr:rowOff>
+      <xdr:rowOff>147240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -782,7 +763,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="211680"/>
-          <a:ext cx="1366200" cy="365040"/>
+          <a:ext cx="1365480" cy="364320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1145,7 +1126,7 @@
       <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="7" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
@@ -1172,7 +1153,7 @@
       <c r="C14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E14" s="7" t="s">
@@ -1199,7 +1180,7 @@
       <c r="C15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="7" t="s">
         <v>35</v>
       </c>
       <c r="E15" s="7" t="s">
@@ -1224,9 +1205,9 @@
         <v>49</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D16" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
       <c r="G16" s="9"/>
@@ -1234,7 +1215,7 @@
         <v>50</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1242,23 +1223,23 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G17" s="7"/>
-      <c r="H17" s="13" t="s">
-        <v>55</v>
+      <c r="H17" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="I17" s="10"/>
     </row>
@@ -1267,22 +1248,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>15</v>
@@ -1294,49 +1275,43 @@
         <v>13</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>65</v>
-      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="9"/>
       <c r="H19" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="10"/>
+      <c r="I19" s="10" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
         <v>14</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="12" t="s">
+      <c r="G20" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>70</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>15</v>
@@ -1348,22 +1323,22 @@
         <v>15</v>
       </c>
       <c r="B21" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="12" t="s">
+      <c r="G21" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>14</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>15</v>
@@ -1375,19 +1350,19 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" s="12" t="s">
+      <c r="F22" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>14</v>
@@ -1402,19 +1377,19 @@
         <v>17</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="F23" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>14</v>
@@ -1429,19 +1404,19 @@
         <v>18</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E24" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="12" t="s">
+      <c r="F24" s="7" t="s">
         <v>84</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>86</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>14</v>
@@ -1456,19 +1431,19 @@
         <v>19</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D25" s="12" t="s">
+      <c r="F25" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>14</v>
@@ -1483,19 +1458,19 @@
         <v>20</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="12" t="s">
+      <c r="F26" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>94</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>14</v>
@@ -1510,19 +1485,19 @@
         <v>21</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E27" s="7" t="s">
+      <c r="F27" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>14</v>
@@ -1530,82 +1505,82 @@
       <c r="H27" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I27" s="11"/>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="n">
         <v>22</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="E28" s="7" t="s">
+      <c r="F28" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="G28" s="9"/>
+      <c r="G28" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="H28" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>50</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="I28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="12" t="s">
+      <c r="F29" s="7" t="s">
         <v>102</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="G29" s="9"/>
       <c r="H29" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I29" s="11"/>
+      <c r="I29" s="10" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="F30" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="G30" s="9"/>
       <c r="H30" s="10" t="s">
         <v>15</v>
       </c>
@@ -1616,49 +1591,49 @@
         <v>25</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E31" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="7" t="s">
+      <c r="F31" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E31" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="G31" s="9" t="s">
-        <v>113</v>
+        <v>33</v>
       </c>
       <c r="H31" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I31" s="10"/>
+      <c r="I31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="n">
         <v>26</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="7" t="s">
+      <c r="G32" s="9" t="s">
         <v>115</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>118</v>
       </c>
       <c r="H32" s="10" t="s">
         <v>15</v>
@@ -1670,29 +1645,55 @@
         <v>27</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F33" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E33" s="7" t="s">
+      <c r="G33" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="H33" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I33" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="C34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H33" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" s="10"/>
-    </row>
-    <row r="1048440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F34" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I34" s="10"/>
+    </row>
     <row r="1048441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>